<commit_message>
ExercicoAulaMarioFIX- Exercicio SQL Injection
</commit_message>
<xml_diff>
--- a/horario_status.xlsx
+++ b/horario_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Slyther1n\Desktop\iefp_formacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5551238B-CF28-40B9-9126-2C08B4BC0458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3382C422-B22A-447F-9E81-3117FEDA27D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A4FA6E67-634F-4E5A-B3C1-BB1AE50EBAF7}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="29">
   <si>
     <t>Código</t>
   </si>
@@ -120,7 +120,7 @@
     <t>Aprovado</t>
   </si>
   <si>
-    <t>Fazer Jogo DVD</t>
+    <t>Trabalho Hands-on-Lab</t>
   </si>
 </sst>
 </file>
@@ -130,7 +130,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,14 +231,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
@@ -877,7 +869,6 @@
     <xf numFmtId="0" fontId="14" fillId="12" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="15" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -893,7 +884,28 @@
     <xf numFmtId="49" fontId="6" fillId="15" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="17" fontId="7" fillId="17" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="7" fillId="17" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="7" fillId="17" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="17" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="17" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="17" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="17" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -906,15 +918,6 @@
     <xf numFmtId="0" fontId="12" fillId="17" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="17" fontId="7" fillId="17" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="7" fillId="17" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="7" fillId="17" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="16" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -930,18 +933,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="17" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="17" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="17" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="17" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Euro" xfId="2" xr:uid="{DD3A81DB-1FA7-4E0F-9A23-1484AF7F90C2}"/>
@@ -1273,14 +1265,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="58.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="3:8" x14ac:dyDescent="0.25">
       <c r="D1" s="14"/>
     </row>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1286,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <v>5089</v>
       </c>
@@ -1307,11 +1299,11 @@
       <c r="F5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="90" t="s">
+      <c r="G5" s="89" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
@@ -1325,7 +1317,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C7" s="4">
         <v>10789</v>
       </c>
@@ -1338,11 +1330,11 @@
       <c r="F7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="90" t="s">
+      <c r="G7" s="89" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C8" s="5">
         <v>5409</v>
       </c>
@@ -1356,7 +1348,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C9" s="6">
         <v>10793</v>
       </c>
@@ -1369,11 +1361,11 @@
       <c r="F9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="90" t="s">
+      <c r="G9" s="89" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C10" s="7">
         <v>10788</v>
       </c>
@@ -1387,7 +1379,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C11" s="8">
         <v>10794</v>
       </c>
@@ -1397,11 +1389,12 @@
       <c r="E11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="84" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="89"/>
+    </row>
+    <row r="12" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C12" s="9">
         <v>10790</v>
       </c>
@@ -1415,7 +1408,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C13" s="10">
         <v>10795</v>
       </c>
@@ -1425,8 +1418,11 @@
       <c r="E13" s="13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F13" s="106" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C14" s="11">
         <v>5425</v>
       </c>
@@ -1436,6 +1432,7 @@
       <c r="E14" s="12" t="s">
         <v>15</v>
       </c>
+      <c r="F14" s="6"/>
     </row>
     <row r="19" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
@@ -1535,17 +1532,17 @@
       </c>
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A20" s="95">
+      <c r="A20" s="90">
         <v>45931</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="93" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="78"/>
       <c r="D20" s="78"/>
       <c r="E20" s="26"/>
       <c r="F20" s="20"/>
-      <c r="G20" s="98" t="s">
+      <c r="G20" s="101" t="s">
         <v>19</v>
       </c>
       <c r="H20" s="28"/>
@@ -1604,13 +1601,13 @@
       </c>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A21" s="96"/>
-      <c r="B21" s="104"/>
+      <c r="A21" s="91"/>
+      <c r="B21" s="94"/>
       <c r="C21" s="51"/>
       <c r="D21" s="51"/>
       <c r="E21" s="22"/>
       <c r="F21" s="17"/>
-      <c r="G21" s="99"/>
+      <c r="G21" s="102"/>
       <c r="H21" s="29"/>
       <c r="I21" s="51"/>
       <c r="J21" s="57">
@@ -1667,13 +1664,13 @@
       </c>
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A22" s="96"/>
-      <c r="B22" s="104"/>
+      <c r="A22" s="91"/>
+      <c r="B22" s="94"/>
       <c r="C22" s="51"/>
       <c r="D22" s="51"/>
       <c r="E22" s="22"/>
       <c r="F22" s="17"/>
-      <c r="G22" s="99"/>
+      <c r="G22" s="102"/>
       <c r="H22" s="29"/>
       <c r="I22" s="51"/>
       <c r="J22" s="57">
@@ -1730,13 +1727,13 @@
       </c>
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A23" s="96"/>
-      <c r="B23" s="104"/>
+      <c r="A23" s="91"/>
+      <c r="B23" s="94"/>
       <c r="C23" s="51"/>
       <c r="D23" s="51"/>
       <c r="E23" s="22"/>
       <c r="F23" s="17"/>
-      <c r="G23" s="99"/>
+      <c r="G23" s="102"/>
       <c r="H23" s="29"/>
       <c r="I23" s="51"/>
       <c r="J23" s="52"/>
@@ -1791,15 +1788,15 @@
       </c>
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A24" s="96"/>
-      <c r="B24" s="103" t="s">
+      <c r="A24" s="91"/>
+      <c r="B24" s="95" t="s">
         <v>21</v>
       </c>
       <c r="C24" s="51"/>
       <c r="D24" s="51"/>
       <c r="E24" s="51"/>
       <c r="F24" s="18"/>
-      <c r="G24" s="99"/>
+      <c r="G24" s="102"/>
       <c r="H24" s="32"/>
       <c r="I24" s="51"/>
       <c r="J24" s="57">
@@ -1854,13 +1851,13 @@
       </c>
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A25" s="96"/>
-      <c r="B25" s="104"/>
+      <c r="A25" s="91"/>
+      <c r="B25" s="94"/>
       <c r="C25" s="51"/>
       <c r="D25" s="51"/>
       <c r="E25" s="51"/>
       <c r="F25" s="19"/>
-      <c r="G25" s="99"/>
+      <c r="G25" s="102"/>
       <c r="H25" s="32"/>
       <c r="I25" s="51"/>
       <c r="J25" s="57">
@@ -1915,13 +1912,13 @@
       </c>
     </row>
     <row r="26" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="97"/>
-      <c r="B26" s="106"/>
+      <c r="A26" s="92"/>
+      <c r="B26" s="96"/>
       <c r="C26" s="55"/>
       <c r="D26" s="55"/>
       <c r="E26" s="55"/>
       <c r="F26" s="21"/>
-      <c r="G26" s="100"/>
+      <c r="G26" s="103"/>
       <c r="H26" s="34"/>
       <c r="I26" s="55"/>
       <c r="J26" s="58">
@@ -1976,10 +1973,10 @@
       </c>
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A27" s="95">
+      <c r="A27" s="90">
         <v>45962</v>
       </c>
-      <c r="B27" s="105" t="s">
+      <c r="B27" s="93" t="s">
         <v>18</v>
       </c>
       <c r="C27" s="20"/>
@@ -2047,8 +2044,8 @@
       <c r="AG27" s="27"/>
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A28" s="96"/>
-      <c r="B28" s="104"/>
+      <c r="A28" s="91"/>
+      <c r="B28" s="94"/>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="49" t="s">
@@ -2114,8 +2111,8 @@
       <c r="AG28" s="25"/>
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A29" s="96"/>
-      <c r="B29" s="104"/>
+      <c r="A29" s="91"/>
+      <c r="B29" s="94"/>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
       <c r="E29" s="49" t="s">
@@ -2181,8 +2178,8 @@
       <c r="AG29" s="25"/>
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A30" s="96"/>
-      <c r="B30" s="104"/>
+      <c r="A30" s="91"/>
+      <c r="B30" s="94"/>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
       <c r="E30" s="49" t="s">
@@ -2248,8 +2245,8 @@
       <c r="AG30" s="25"/>
     </row>
     <row r="31" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A31" s="96"/>
-      <c r="B31" s="103" t="s">
+      <c r="A31" s="91"/>
+      <c r="B31" s="95" t="s">
         <v>21</v>
       </c>
       <c r="C31" s="18"/>
@@ -2301,8 +2298,8 @@
       <c r="AG31" s="25"/>
     </row>
     <row r="32" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A32" s="96"/>
-      <c r="B32" s="104"/>
+      <c r="A32" s="91"/>
+      <c r="B32" s="94"/>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
       <c r="E32" s="51"/>
@@ -2352,8 +2349,8 @@
       <c r="AG32" s="25"/>
     </row>
     <row r="33" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="97"/>
-      <c r="B33" s="106"/>
+      <c r="A33" s="92"/>
+      <c r="B33" s="96"/>
       <c r="C33" s="21"/>
       <c r="D33" s="21"/>
       <c r="E33" s="55"/>
@@ -2403,13 +2400,13 @@
       <c r="AG33" s="35"/>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A34" s="96">
+      <c r="A34" s="91">
         <v>45992</v>
       </c>
-      <c r="B34" s="104" t="s">
+      <c r="B34" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="97" t="s">
         <v>19</v>
       </c>
       <c r="D34" s="69" t="s">
@@ -2424,7 +2421,7 @@
       </c>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
-      <c r="J34" s="91" t="s">
+      <c r="J34" s="97" t="s">
         <v>19</v>
       </c>
       <c r="K34" s="69" t="s">
@@ -2449,7 +2446,7 @@
       <c r="X34" s="36"/>
       <c r="Y34" s="36"/>
       <c r="Z34" s="36"/>
-      <c r="AA34" s="91" t="s">
+      <c r="AA34" s="97" t="s">
         <v>24</v>
       </c>
       <c r="AB34" s="36"/>
@@ -2460,9 +2457,9 @@
       <c r="AG34" s="36"/>
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A35" s="96"/>
-      <c r="B35" s="104"/>
-      <c r="C35" s="91"/>
+      <c r="A35" s="91"/>
+      <c r="B35" s="94"/>
+      <c r="C35" s="97"/>
       <c r="D35" s="47" t="s">
         <v>22</v>
       </c>
@@ -2475,7 +2472,7 @@
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
-      <c r="J35" s="91"/>
+      <c r="J35" s="97"/>
       <c r="K35" s="47" t="s">
         <v>22</v>
       </c>
@@ -2498,7 +2495,7 @@
       <c r="X35" s="36"/>
       <c r="Y35" s="36"/>
       <c r="Z35" s="36"/>
-      <c r="AA35" s="91"/>
+      <c r="AA35" s="97"/>
       <c r="AB35" s="36"/>
       <c r="AC35" s="17"/>
       <c r="AD35" s="17"/>
@@ -2507,9 +2504,9 @@
       <c r="AG35" s="36"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A36" s="96"/>
-      <c r="B36" s="104"/>
-      <c r="C36" s="91"/>
+      <c r="A36" s="91"/>
+      <c r="B36" s="94"/>
+      <c r="C36" s="97"/>
       <c r="D36" s="47" t="s">
         <v>22</v>
       </c>
@@ -2522,7 +2519,7 @@
       </c>
       <c r="H36" s="17"/>
       <c r="I36" s="17"/>
-      <c r="J36" s="91"/>
+      <c r="J36" s="97"/>
       <c r="K36" s="47" t="s">
         <v>22</v>
       </c>
@@ -2545,7 +2542,7 @@
       <c r="X36" s="36"/>
       <c r="Y36" s="36"/>
       <c r="Z36" s="36"/>
-      <c r="AA36" s="91"/>
+      <c r="AA36" s="97"/>
       <c r="AB36" s="36"/>
       <c r="AC36" s="17"/>
       <c r="AD36" s="17"/>
@@ -2554,9 +2551,9 @@
       <c r="AG36" s="36"/>
     </row>
     <row r="37" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A37" s="96"/>
-      <c r="B37" s="104"/>
-      <c r="C37" s="91"/>
+      <c r="A37" s="91"/>
+      <c r="B37" s="94"/>
+      <c r="C37" s="97"/>
       <c r="D37" s="47" t="s">
         <v>22</v>
       </c>
@@ -2569,7 +2566,7 @@
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
-      <c r="J37" s="91"/>
+      <c r="J37" s="97"/>
       <c r="K37" s="48" t="s">
         <v>23</v>
       </c>
@@ -2592,7 +2589,7 @@
       <c r="X37" s="36"/>
       <c r="Y37" s="36"/>
       <c r="Z37" s="36"/>
-      <c r="AA37" s="91"/>
+      <c r="AA37" s="97"/>
       <c r="AB37" s="36"/>
       <c r="AC37" s="17"/>
       <c r="AD37" s="17"/>
@@ -2601,11 +2598,11 @@
       <c r="AG37" s="36"/>
     </row>
     <row r="38" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A38" s="96"/>
-      <c r="B38" s="103" t="s">
+      <c r="A38" s="91"/>
+      <c r="B38" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="91"/>
+      <c r="C38" s="97"/>
       <c r="D38" s="53"/>
       <c r="E38" s="60">
         <v>10793</v>
@@ -2616,7 +2613,7 @@
       </c>
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
-      <c r="J38" s="91"/>
+      <c r="J38" s="97"/>
       <c r="K38" s="53"/>
       <c r="L38" s="63">
         <v>10794</v>
@@ -2637,7 +2634,7 @@
       <c r="X38" s="32"/>
       <c r="Y38" s="32"/>
       <c r="Z38" s="32"/>
-      <c r="AA38" s="91"/>
+      <c r="AA38" s="97"/>
       <c r="AB38" s="32"/>
       <c r="AC38" s="18"/>
       <c r="AD38" s="18"/>
@@ -2646,9 +2643,9 @@
       <c r="AG38" s="32"/>
     </row>
     <row r="39" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A39" s="96"/>
-      <c r="B39" s="104"/>
-      <c r="C39" s="91"/>
+      <c r="A39" s="91"/>
+      <c r="B39" s="94"/>
+      <c r="C39" s="97"/>
       <c r="D39" s="53"/>
       <c r="E39" s="60">
         <v>10793</v>
@@ -2659,7 +2656,7 @@
       </c>
       <c r="H39" s="19"/>
       <c r="I39" s="19"/>
-      <c r="J39" s="91"/>
+      <c r="J39" s="97"/>
       <c r="K39" s="53"/>
       <c r="L39" s="63">
         <v>10794</v>
@@ -2680,7 +2677,7 @@
       <c r="X39" s="32"/>
       <c r="Y39" s="32"/>
       <c r="Z39" s="32"/>
-      <c r="AA39" s="91"/>
+      <c r="AA39" s="97"/>
       <c r="AB39" s="32"/>
       <c r="AC39" s="19"/>
       <c r="AD39" s="19"/>
@@ -2689,9 +2686,9 @@
       <c r="AG39" s="32"/>
     </row>
     <row r="40" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="96"/>
-      <c r="B40" s="104"/>
-      <c r="C40" s="91"/>
+      <c r="A40" s="91"/>
+      <c r="B40" s="94"/>
+      <c r="C40" s="97"/>
       <c r="D40" s="56"/>
       <c r="E40" s="60">
         <v>10793</v>
@@ -2702,7 +2699,7 @@
       </c>
       <c r="H40" s="33"/>
       <c r="I40" s="33"/>
-      <c r="J40" s="91"/>
+      <c r="J40" s="97"/>
       <c r="K40" s="54"/>
       <c r="L40" s="66">
         <v>10794</v>
@@ -2723,7 +2720,7 @@
       <c r="X40" s="54"/>
       <c r="Y40" s="54"/>
       <c r="Z40" s="54"/>
-      <c r="AA40" s="91"/>
+      <c r="AA40" s="97"/>
       <c r="AB40" s="54"/>
       <c r="AC40" s="33"/>
       <c r="AD40" s="33"/>
@@ -2732,13 +2729,13 @@
       <c r="AG40" s="54"/>
     </row>
     <row r="41" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A41" s="95">
+      <c r="A41" s="90">
         <v>46023</v>
       </c>
-      <c r="B41" s="105" t="s">
+      <c r="B41" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C41" s="101" t="s">
+      <c r="C41" s="104" t="s">
         <v>19</v>
       </c>
       <c r="D41" s="37"/>
@@ -2748,8 +2745,8 @@
       <c r="H41" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="I41" s="85"/>
-      <c r="J41" s="85"/>
+      <c r="I41" s="84"/>
+      <c r="J41" s="84"/>
       <c r="K41" s="37"/>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
@@ -2763,7 +2760,7 @@
       <c r="Q41" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="R41" s="88" t="s">
+      <c r="R41" s="87" t="s">
         <v>23</v>
       </c>
       <c r="S41" s="20"/>
@@ -2785,7 +2782,7 @@
       <c r="AC41" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="AD41" s="87"/>
+      <c r="AD41" s="86"/>
       <c r="AE41" s="65">
         <v>10794</v>
       </c>
@@ -2795,9 +2792,9 @@
       <c r="AG41" s="20"/>
     </row>
     <row r="42" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A42" s="96"/>
-      <c r="B42" s="104"/>
-      <c r="C42" s="91"/>
+      <c r="A42" s="91"/>
+      <c r="B42" s="94"/>
+      <c r="C42" s="97"/>
       <c r="D42" s="36"/>
       <c r="E42" s="17"/>
       <c r="F42" s="17"/>
@@ -2805,8 +2802,8 @@
       <c r="H42" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="I42" s="86"/>
-      <c r="J42" s="86"/>
+      <c r="I42" s="85"/>
+      <c r="J42" s="85"/>
       <c r="K42" s="36"/>
       <c r="L42" s="17"/>
       <c r="M42" s="17"/>
@@ -2842,7 +2839,7 @@
       <c r="AC42" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="AD42" s="89"/>
+      <c r="AD42" s="88"/>
       <c r="AE42" s="63">
         <v>10794</v>
       </c>
@@ -2852,9 +2849,9 @@
       <c r="AG42" s="17"/>
     </row>
     <row r="43" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A43" s="96"/>
-      <c r="B43" s="104"/>
-      <c r="C43" s="91"/>
+      <c r="A43" s="91"/>
+      <c r="B43" s="94"/>
+      <c r="C43" s="97"/>
       <c r="D43" s="36"/>
       <c r="E43" s="17"/>
       <c r="F43" s="17"/>
@@ -2862,8 +2859,8 @@
       <c r="H43" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="I43" s="86"/>
-      <c r="J43" s="86"/>
+      <c r="I43" s="85"/>
+      <c r="J43" s="85"/>
       <c r="K43" s="36"/>
       <c r="L43" s="17"/>
       <c r="M43" s="17"/>
@@ -2899,7 +2896,7 @@
       <c r="AC43" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="AD43" s="89"/>
+      <c r="AD43" s="88"/>
       <c r="AE43" s="63">
         <v>10794</v>
       </c>
@@ -2909,9 +2906,9 @@
       <c r="AG43" s="17"/>
     </row>
     <row r="44" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A44" s="96"/>
-      <c r="B44" s="104"/>
-      <c r="C44" s="91"/>
+      <c r="A44" s="91"/>
+      <c r="B44" s="94"/>
+      <c r="C44" s="97"/>
       <c r="D44" s="36"/>
       <c r="E44" s="17"/>
       <c r="F44" s="17"/>
@@ -2919,8 +2916,8 @@
       <c r="H44" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="I44" s="86"/>
-      <c r="J44" s="86"/>
+      <c r="I44" s="85"/>
+      <c r="J44" s="85"/>
       <c r="K44" s="36"/>
       <c r="L44" s="17"/>
       <c r="M44" s="17"/>
@@ -2956,7 +2953,7 @@
       <c r="AC44" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="AD44" s="89"/>
+      <c r="AD44" s="88"/>
       <c r="AE44" s="63">
         <v>10794</v>
       </c>
@@ -2966,11 +2963,11 @@
       <c r="AG44" s="17"/>
     </row>
     <row r="45" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A45" s="96"/>
-      <c r="B45" s="103" t="s">
+      <c r="A45" s="91"/>
+      <c r="B45" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="C45" s="91"/>
+      <c r="C45" s="97"/>
       <c r="D45" s="32"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -3013,7 +3010,7 @@
       <c r="AC45" s="63">
         <v>10794</v>
       </c>
-      <c r="AD45" s="89"/>
+      <c r="AD45" s="88"/>
       <c r="AE45" s="63">
         <v>10794</v>
       </c>
@@ -3023,9 +3020,9 @@
       <c r="AG45" s="18"/>
     </row>
     <row r="46" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A46" s="96"/>
-      <c r="B46" s="104"/>
-      <c r="C46" s="91"/>
+      <c r="A46" s="91"/>
+      <c r="B46" s="94"/>
+      <c r="C46" s="97"/>
       <c r="D46" s="32"/>
       <c r="E46" s="19"/>
       <c r="F46" s="19"/>
@@ -3078,9 +3075,9 @@
       <c r="AG46" s="19"/>
     </row>
     <row r="47" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="97"/>
-      <c r="B47" s="106"/>
-      <c r="C47" s="102"/>
+      <c r="A47" s="92"/>
+      <c r="B47" s="96"/>
+      <c r="C47" s="105"/>
       <c r="D47" s="34"/>
       <c r="E47" s="21"/>
       <c r="F47" s="21"/>
@@ -3131,10 +3128,10 @@
       <c r="AG47" s="21"/>
     </row>
     <row r="48" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A48" s="95">
+      <c r="A48" s="90">
         <v>46054</v>
       </c>
-      <c r="B48" s="105" t="s">
+      <c r="B48" s="93" t="s">
         <v>18</v>
       </c>
       <c r="C48" s="39"/>
@@ -3163,7 +3160,7 @@
       <c r="P48" s="39"/>
       <c r="Q48" s="39"/>
       <c r="R48" s="37"/>
-      <c r="S48" s="92" t="s">
+      <c r="S48" s="98" t="s">
         <v>26</v>
       </c>
       <c r="T48" s="82">
@@ -3190,8 +3187,8 @@
       <c r="AG48" s="43"/>
     </row>
     <row r="49" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A49" s="96"/>
-      <c r="B49" s="104"/>
+      <c r="A49" s="91"/>
+      <c r="B49" s="94"/>
       <c r="C49" s="40"/>
       <c r="D49" s="36"/>
       <c r="E49" s="68" t="s">
@@ -3218,7 +3215,7 @@
       <c r="P49" s="40"/>
       <c r="Q49" s="40"/>
       <c r="R49" s="36"/>
-      <c r="S49" s="93"/>
+      <c r="S49" s="99"/>
       <c r="T49" s="67">
         <v>5425</v>
       </c>
@@ -3243,8 +3240,8 @@
       <c r="AG49" s="44"/>
     </row>
     <row r="50" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A50" s="96"/>
-      <c r="B50" s="104"/>
+      <c r="A50" s="91"/>
+      <c r="B50" s="94"/>
       <c r="C50" s="40"/>
       <c r="D50" s="36"/>
       <c r="E50" s="68" t="s">
@@ -3271,7 +3268,7 @@
       <c r="P50" s="40"/>
       <c r="Q50" s="40"/>
       <c r="R50" s="36"/>
-      <c r="S50" s="93"/>
+      <c r="S50" s="99"/>
       <c r="T50" s="67">
         <v>5425</v>
       </c>
@@ -3296,8 +3293,8 @@
       <c r="AG50" s="44"/>
     </row>
     <row r="51" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A51" s="96"/>
-      <c r="B51" s="104"/>
+      <c r="A51" s="91"/>
+      <c r="B51" s="94"/>
       <c r="C51" s="40"/>
       <c r="D51" s="36"/>
       <c r="E51" s="68" t="s">
@@ -3324,7 +3321,7 @@
       <c r="P51" s="40"/>
       <c r="Q51" s="40"/>
       <c r="R51" s="36"/>
-      <c r="S51" s="93"/>
+      <c r="S51" s="99"/>
       <c r="T51" s="67">
         <v>5425</v>
       </c>
@@ -3349,8 +3346,8 @@
       <c r="AG51" s="44"/>
     </row>
     <row r="52" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A52" s="96"/>
-      <c r="B52" s="103" t="s">
+      <c r="A52" s="91"/>
+      <c r="B52" s="95" t="s">
         <v>21</v>
       </c>
       <c r="C52" s="41"/>
@@ -3379,7 +3376,7 @@
       <c r="P52" s="41"/>
       <c r="Q52" s="41"/>
       <c r="R52" s="32"/>
-      <c r="S52" s="93"/>
+      <c r="S52" s="99"/>
       <c r="T52" s="67">
         <v>5425</v>
       </c>
@@ -3404,8 +3401,8 @@
       <c r="AG52" s="45"/>
     </row>
     <row r="53" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A53" s="96"/>
-      <c r="B53" s="104"/>
+      <c r="A53" s="91"/>
+      <c r="B53" s="94"/>
       <c r="C53" s="41"/>
       <c r="D53" s="32"/>
       <c r="E53" s="63">
@@ -3432,7 +3429,7 @@
       <c r="P53" s="41"/>
       <c r="Q53" s="41"/>
       <c r="R53" s="32"/>
-      <c r="S53" s="93"/>
+      <c r="S53" s="99"/>
       <c r="T53" s="67">
         <v>5425</v>
       </c>
@@ -3457,8 +3454,8 @@
       <c r="AG53" s="45"/>
     </row>
     <row r="54" spans="1:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="97"/>
-      <c r="B54" s="106"/>
+      <c r="A54" s="92"/>
+      <c r="B54" s="96"/>
       <c r="C54" s="42"/>
       <c r="D54" s="34"/>
       <c r="E54" s="64">
@@ -3485,7 +3482,7 @@
       <c r="P54" s="42"/>
       <c r="Q54" s="42"/>
       <c r="R54" s="34"/>
-      <c r="S54" s="94"/>
+      <c r="S54" s="100"/>
       <c r="T54" s="34"/>
       <c r="U54" s="83">
         <v>5425</v>
@@ -3509,11 +3506,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A41:A47"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="A48:A54"/>
-    <mergeCell ref="J34:J40"/>
     <mergeCell ref="AA34:AA40"/>
     <mergeCell ref="C34:C40"/>
     <mergeCell ref="S48:S54"/>
@@ -3530,8 +3522,13 @@
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="B48:B51"/>
     <mergeCell ref="B52:B54"/>
+    <mergeCell ref="A41:A47"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="A48:A54"/>
+    <mergeCell ref="J34:J40"/>
   </mergeCells>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="C6" numberStoredAsText="1"/>

</xml_diff>